<commit_message>
backup updated labeled data
</commit_message>
<xml_diff>
--- a/CategorySlowTestsIssuesFromGithub.xlsx
+++ b/CategorySlowTestsIssuesFromGithub.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xutongliu/LLM/SlowTestOpt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B2BF11-A659-A74E-89AE-961774C3B562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C5B157-2D72-C344-96AF-86B8D0CD4286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="500" windowWidth="38400" windowHeight="19860" xr2:uid="{6939473A-5637-5F49-BCB2-3074E35B3208}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17640" xr2:uid="{6939473A-5637-5F49-BCB2-3074E35B3208}"/>
   </bookViews>
   <sheets>
     <sheet name="slow_test_issues" sheetId="2" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6490" uniqueCount="3914">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6550" uniqueCount="3947">
   <si>
     <t>repo_full_name</t>
   </si>
@@ -12093,12 +12093,203 @@
   <si>
     <t>【Hypothesis】Optimize slow benchmark tests by refactoring them to use Hypothesis property-based testing instead of exhaustive case enumeration, reducing test execution time from 30-48 seconds per test to a fraction of that while maintaining or improving test coverage through intelligent test case generation.</t>
   </si>
+  <si>
+    <t>This issue is about restructuring a GitHub Actions workflow to add a manual approval step, not about tests being too slow to execute.</t>
+  </si>
+  <si>
+    <t>This issue is about an integration test (test_can_bundle_configured_catalogs) that is extremely slow, taking 19-27 minutes to execute when it should be much faster, eventually causing timeouts.</t>
+  </si>
+  <si>
+    <t>https://github.com/DataBiosphere/azul/pull/5057</t>
+  </si>
+  <si>
+    <t>Reducing redundant function calls</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> This issue is about the forward model runner hanging after completing (a connection/communication problem), not about the tests or processes being too slow to execute.</t>
+  </si>
+  <si>
+    <t>This issue is about incorrect Python logging configuration in library code that interferes with user logging settings, not about tests being too slow to execute.</t>
+  </si>
+  <si>
+    <t>This issue is about reorganizing the test directory structure for better code organization, not about tests being too slow to execute.</t>
+  </si>
+  <si>
+    <t>This issue is about a runtime error/regression in PyTorch 2.8 RC where tests fail with a "last dimension must be contiguous" error, not about tests being too slow to execute.</t>
+  </si>
+  <si>
+    <t>not related</t>
+  </si>
+  <si>
+    <t>This issue is about avoiding slow UI testing by using mock clients instead of making actual API endpoint calls, which the author explicitly states are "slow" and risky when testing frequently.</t>
+  </si>
+  <si>
+    <t>https://github.com/supreme-gg-gg/instagram-cli/pull/137</t>
+  </si>
+  <si>
+    <t>Hybrid: Major feature with test refactoring</t>
+  </si>
+  <si>
+    <t>“New mocking system that is pretty simple but can reduce API calls during development”</t>
+  </si>
+  <si>
+    <t>Title is clear</t>
+  </si>
+  <si>
+    <r>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> pytest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF383A42"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">xdist for parallel execution </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF383A42"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Split tests into separate workflows </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF383A42"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Remove unnecessary builds (Horovod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF383A42"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> TensorFlow)</t>
+    </r>
+  </si>
+  <si>
+    <t>Dependency update</t>
+  </si>
+  <si>
+    <t>install the dependencies with uv instead of pip</t>
+  </si>
+  <si>
+    <t>https://github.com/interTwin-eu/itwinai/pull/293</t>
+  </si>
+  <si>
+    <t>This issue is about adding the ability to pass additional pytest options (like test filtering and plugin configuration) to mutation testing runs, not about tests being too slow to execute.</t>
+  </si>
+  <si>
+    <t>https://github.com/causify-ai/helpers/pull/422</t>
+  </si>
+  <si>
+    <t>Not Related</t>
+  </si>
+  <si>
+    <t>To add new unit test for imporve code coverage</t>
+  </si>
+  <si>
+    <t>workflow refacotring：This issue is about changing the trigger mechanism for slow tests from commit messages to GitHub environment approval, not about the tests themselves being too slow.</t>
+  </si>
+  <si>
+    <t>Bug：This issue is about insufficient numerical accuracy in geminal calculations causing test failures, not about tests being too slow to execute.</t>
+  </si>
+  <si>
+    <t>This issue's main complaint is that HTTP requests in tests can fail for various reasons including "w3id is feeling slow that day", causing CI failures. The issue explicitly mentions slowness as one of the problems with real HTTP requests in tests.</t>
+  </si>
+  <si>
+    <t>https://github.com/Jelly-RDF/pyjelly/pull/235</t>
+  </si>
+  <si>
+    <t>Add HTTP mocking for example tests to avoid real network requests, improve test stability and speed, eliminate external dependencies, and adopt a 'good enough' strategy that accepts some boundary cases not being perfectly handled.</t>
+  </si>
+  <si>
+    <t>This issue is about a disabled/failing test on the XPU platform, not about the test being too slow to execute.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> This issue is about enabling database migrations during CI testing to catch migration problems earlier. </t>
+  </si>
+  <si>
+    <t>disable failed test</t>
+  </si>
+  <si>
+    <t>This issue's main complaint includes that "testing against the live Dify API can be slow, expensive, and unpredictable." The proposal explicitly aims to achieve "Faster Testing: Run tests locally without API dependencies" by adding mock infrastructure to avoid slow API testing.</t>
+  </si>
+  <si>
+    <t>https://github.com/laipz8200/anime-librarian/pull/21</t>
+  </si>
+  <si>
+    <t>Add Mock Dify Server and Fixtures, full integration tests, automated linting scripts, Makefile commands,</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -12166,6 +12357,13 @@
       <name val="Arial Unicode MS"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF383A42"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -12188,7 +12386,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -12203,6 +12401,7 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -24454,7 +24653,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="209" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>1130</v>
       </c>
@@ -24507,7 +24706,7 @@
         <v>1135</v>
       </c>
     </row>
-    <row r="210" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>1136</v>
       </c>
@@ -24560,7 +24759,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="211" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>1142</v>
       </c>
@@ -24613,7 +24812,7 @@
         <v>1146</v>
       </c>
     </row>
-    <row r="212" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>1147</v>
       </c>
@@ -24666,7 +24865,7 @@
         <v>1152</v>
       </c>
     </row>
-    <row r="213" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>1153</v>
       </c>
@@ -24719,7 +24918,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="214" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>1159</v>
       </c>
@@ -24750,6 +24949,9 @@
       <c r="J214" t="s">
         <v>1161</v>
       </c>
+      <c r="K214" t="s">
+        <v>3914</v>
+      </c>
       <c r="L214" s="7" t="s">
         <v>1162</v>
       </c>
@@ -24771,8 +24973,11 @@
       <c r="R214" t="s">
         <v>1163</v>
       </c>
-    </row>
-    <row r="215" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+      <c r="T214" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="215" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>1164</v>
       </c>
@@ -24803,6 +25008,9 @@
       <c r="J215" t="s">
         <v>1166</v>
       </c>
+      <c r="K215" t="s">
+        <v>3915</v>
+      </c>
       <c r="L215" s="7" t="s">
         <v>1167</v>
       </c>
@@ -24824,8 +25032,20 @@
       <c r="R215" t="s">
         <v>1169</v>
       </c>
-    </row>
-    <row r="216" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S215" s="5" t="s">
+        <v>3916</v>
+      </c>
+      <c r="T215" t="s">
+        <v>3869</v>
+      </c>
+      <c r="U215" t="s">
+        <v>3774</v>
+      </c>
+      <c r="V215" t="s">
+        <v>3917</v>
+      </c>
+    </row>
+    <row r="216" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>1170</v>
       </c>
@@ -24878,7 +25098,7 @@
         <v>1174</v>
       </c>
     </row>
-    <row r="217" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>1175</v>
       </c>
@@ -24931,7 +25151,7 @@
         <v>1179</v>
       </c>
     </row>
-    <row r="218" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>971</v>
       </c>
@@ -24984,7 +25204,7 @@
         <v>1183</v>
       </c>
     </row>
-    <row r="219" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>809</v>
       </c>
@@ -25037,7 +25257,7 @@
         <v>1187</v>
       </c>
     </row>
-    <row r="220" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>1188</v>
       </c>
@@ -25090,7 +25310,7 @@
         <v>1192</v>
       </c>
     </row>
-    <row r="221" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>1193</v>
       </c>
@@ -25143,7 +25363,7 @@
         <v>1198</v>
       </c>
     </row>
-    <row r="222" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>1199</v>
       </c>
@@ -25196,7 +25416,7 @@
         <v>1204</v>
       </c>
     </row>
-    <row r="223" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>1205</v>
       </c>
@@ -25249,7 +25469,7 @@
         <v>1210</v>
       </c>
     </row>
-    <row r="224" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>1211</v>
       </c>
@@ -25302,7 +25522,7 @@
         <v>1215</v>
       </c>
     </row>
-    <row r="225" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>1216</v>
       </c>
@@ -25355,7 +25575,7 @@
         <v>1221</v>
       </c>
     </row>
-    <row r="226" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>455</v>
       </c>
@@ -25408,7 +25628,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="227" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>1225</v>
       </c>
@@ -25461,7 +25681,7 @@
         <v>1230</v>
       </c>
     </row>
-    <row r="228" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>1231</v>
       </c>
@@ -25514,7 +25734,7 @@
         <v>1236</v>
       </c>
     </row>
-    <row r="229" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>184</v>
       </c>
@@ -25567,7 +25787,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="230" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>1239</v>
       </c>
@@ -25620,7 +25840,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="231" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>1245</v>
       </c>
@@ -25673,7 +25893,7 @@
         <v>1251</v>
       </c>
     </row>
-    <row r="232" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:20" ht="17" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>346</v>
       </c>
@@ -25704,6 +25924,9 @@
       <c r="J232" t="s">
         <v>1252</v>
       </c>
+      <c r="K232" t="s">
+        <v>3918</v>
+      </c>
       <c r="L232" s="7" t="s">
         <v>1253</v>
       </c>
@@ -25725,8 +25948,11 @@
       <c r="R232" t="s">
         <v>1254</v>
       </c>
-    </row>
-    <row r="233" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="T232" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="233" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>1255</v>
       </c>
@@ -25779,7 +26005,7 @@
         <v>1260</v>
       </c>
     </row>
-    <row r="234" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:20" ht="34" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>1261</v>
       </c>
@@ -25810,7 +26036,10 @@
       <c r="J234" t="s">
         <v>1263</v>
       </c>
-      <c r="L234" s="6" t="s">
+      <c r="K234" t="s">
+        <v>3919</v>
+      </c>
+      <c r="L234" s="7" t="s">
         <v>1264</v>
       </c>
       <c r="M234" t="s">
@@ -25831,8 +26060,11 @@
       <c r="R234" t="s">
         <v>1265</v>
       </c>
-    </row>
-    <row r="235" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="T234" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="235" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>483</v>
       </c>
@@ -25885,7 +26117,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="236" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>1269</v>
       </c>
@@ -25938,7 +26170,7 @@
         <v>1273</v>
       </c>
     </row>
-    <row r="237" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>1274</v>
       </c>
@@ -25991,7 +26223,7 @@
         <v>1278</v>
       </c>
     </row>
-    <row r="238" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>1279</v>
       </c>
@@ -26044,7 +26276,7 @@
         <v>1284</v>
       </c>
     </row>
-    <row r="239" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>1285</v>
       </c>
@@ -26097,7 +26329,7 @@
         <v>1289</v>
       </c>
     </row>
-    <row r="240" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>1290</v>
       </c>
@@ -26150,7 +26382,7 @@
         <v>1294</v>
       </c>
     </row>
-    <row r="241" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>1295</v>
       </c>
@@ -26203,7 +26435,7 @@
         <v>1300</v>
       </c>
     </row>
-    <row r="242" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>1301</v>
       </c>
@@ -26256,7 +26488,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="243" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>1306</v>
       </c>
@@ -26309,7 +26541,7 @@
         <v>1312</v>
       </c>
     </row>
-    <row r="244" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>1313</v>
       </c>
@@ -26362,7 +26594,7 @@
         <v>1318</v>
       </c>
     </row>
-    <row r="245" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>1319</v>
       </c>
@@ -26393,7 +26625,10 @@
       <c r="J245" t="s">
         <v>1321</v>
       </c>
-      <c r="L245" s="6" t="s">
+      <c r="K245" t="s">
+        <v>3920</v>
+      </c>
+      <c r="L245" s="7" t="s">
         <v>1322</v>
       </c>
       <c r="M245" t="s">
@@ -26414,8 +26649,11 @@
       <c r="R245" t="s">
         <v>1323</v>
       </c>
-    </row>
-    <row r="246" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="T245" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="246" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>903</v>
       </c>
@@ -26468,7 +26706,7 @@
         <v>1327</v>
       </c>
     </row>
-    <row r="247" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>449</v>
       </c>
@@ -26499,7 +26737,10 @@
       <c r="J247" t="s">
         <v>1328</v>
       </c>
-      <c r="L247" s="6" t="s">
+      <c r="K247" t="s">
+        <v>3921</v>
+      </c>
+      <c r="L247" s="7" t="s">
         <v>1329</v>
       </c>
       <c r="M247" t="s">
@@ -26520,8 +26761,11 @@
       <c r="R247" t="s">
         <v>1331</v>
       </c>
-    </row>
-    <row r="248" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="T247" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="248" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>529</v>
       </c>
@@ -26574,7 +26818,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="249" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>1335</v>
       </c>
@@ -26605,7 +26849,10 @@
       <c r="J249" t="s">
         <v>1337</v>
       </c>
-      <c r="L249" s="6" t="s">
+      <c r="K249" t="s">
+        <v>3922</v>
+      </c>
+      <c r="L249" s="7" t="s">
         <v>1338</v>
       </c>
       <c r="M249" t="s">
@@ -26626,8 +26873,11 @@
       <c r="R249" t="s">
         <v>1339</v>
       </c>
-    </row>
-    <row r="250" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+      <c r="T249" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="250" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>1340</v>
       </c>
@@ -26658,7 +26908,10 @@
       <c r="J250" t="s">
         <v>1342</v>
       </c>
-      <c r="L250" s="6" t="s">
+      <c r="K250" t="s">
+        <v>3923</v>
+      </c>
+      <c r="L250" s="7" t="s">
         <v>1343</v>
       </c>
       <c r="M250" t="s">
@@ -26679,8 +26932,20 @@
       <c r="R250" t="s">
         <v>1345</v>
       </c>
-    </row>
-    <row r="251" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S250" s="5" t="s">
+        <v>3924</v>
+      </c>
+      <c r="T250" t="s">
+        <v>3869</v>
+      </c>
+      <c r="U250" t="s">
+        <v>3925</v>
+      </c>
+      <c r="V250" t="s">
+        <v>3926</v>
+      </c>
+    </row>
+    <row r="251" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>1346</v>
       </c>
@@ -26733,7 +26998,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="252" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>103</v>
       </c>
@@ -26786,7 +27051,7 @@
         <v>1354</v>
       </c>
     </row>
-    <row r="253" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>1355</v>
       </c>
@@ -26839,7 +27104,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="254" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>1360</v>
       </c>
@@ -26892,7 +27157,7 @@
         <v>1365</v>
       </c>
     </row>
-    <row r="255" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>1366</v>
       </c>
@@ -26945,7 +27210,7 @@
         <v>1371</v>
       </c>
     </row>
-    <row r="256" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>1372</v>
       </c>
@@ -26998,7 +27263,7 @@
         <v>1377</v>
       </c>
     </row>
-    <row r="257" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>1378</v>
       </c>
@@ -27051,7 +27316,7 @@
         <v>1383</v>
       </c>
     </row>
-    <row r="258" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>1384</v>
       </c>
@@ -27104,7 +27369,7 @@
         <v>1389</v>
       </c>
     </row>
-    <row r="259" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:24" ht="34" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>1390</v>
       </c>
@@ -27135,7 +27400,10 @@
       <c r="J259" t="s">
         <v>1392</v>
       </c>
-      <c r="L259" s="6" t="s">
+      <c r="K259" t="s">
+        <v>3927</v>
+      </c>
+      <c r="L259" s="7" t="s">
         <v>1393</v>
       </c>
       <c r="M259" t="s">
@@ -27156,8 +27424,26 @@
       <c r="R259" t="s">
         <v>1395</v>
       </c>
-    </row>
-    <row r="260" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+      <c r="S259" s="5" t="s">
+        <v>3931</v>
+      </c>
+      <c r="T259" t="s">
+        <v>3869</v>
+      </c>
+      <c r="U259" t="s">
+        <v>3873</v>
+      </c>
+      <c r="V259" s="10" t="s">
+        <v>3928</v>
+      </c>
+      <c r="W259" t="s">
+        <v>3929</v>
+      </c>
+      <c r="X259" t="s">
+        <v>3930</v>
+      </c>
+    </row>
+    <row r="260" spans="1:24" ht="34" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>1396</v>
       </c>
@@ -27188,7 +27474,10 @@
       <c r="J260" t="s">
         <v>1398</v>
       </c>
-      <c r="L260" s="6" t="s">
+      <c r="K260" t="s">
+        <v>3932</v>
+      </c>
+      <c r="L260" s="7" t="s">
         <v>1399</v>
       </c>
       <c r="M260" t="s">
@@ -27209,8 +27498,11 @@
       <c r="R260" t="s">
         <v>1400</v>
       </c>
-    </row>
-    <row r="261" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="T260" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="261" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
         <v>1401</v>
       </c>
@@ -27263,7 +27555,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="262" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
         <v>1406</v>
       </c>
@@ -27316,7 +27608,7 @@
         <v>1411</v>
       </c>
     </row>
-    <row r="263" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
         <v>1412</v>
       </c>
@@ -27369,7 +27661,7 @@
         <v>1416</v>
       </c>
     </row>
-    <row r="264" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
         <v>1417</v>
       </c>
@@ -27422,7 +27714,7 @@
         <v>1422</v>
       </c>
     </row>
-    <row r="265" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
         <v>1423</v>
       </c>
@@ -27475,7 +27767,7 @@
         <v>1428</v>
       </c>
     </row>
-    <row r="266" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
         <v>1429</v>
       </c>
@@ -27528,7 +27820,7 @@
         <v>1433</v>
       </c>
     </row>
-    <row r="267" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
         <v>1434</v>
       </c>
@@ -27581,7 +27873,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="268" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
         <v>881</v>
       </c>
@@ -27634,7 +27926,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="269" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:24" ht="34" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
         <v>1444</v>
       </c>
@@ -27665,7 +27957,10 @@
       <c r="J269" t="s">
         <v>1446</v>
       </c>
-      <c r="L269" s="6" t="s">
+      <c r="K269" t="s">
+        <v>3935</v>
+      </c>
+      <c r="L269" s="7" t="s">
         <v>1447</v>
       </c>
       <c r="M269" t="s">
@@ -27686,8 +27981,14 @@
       <c r="R269" t="s">
         <v>1448</v>
       </c>
-    </row>
-    <row r="270" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S269" s="5" t="s">
+        <v>3933</v>
+      </c>
+      <c r="T269" t="s">
+        <v>3934</v>
+      </c>
+    </row>
+    <row r="270" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
         <v>1449</v>
       </c>
@@ -27740,7 +28041,7 @@
         <v>1454</v>
       </c>
     </row>
-    <row r="271" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
       <c r="A271" t="s">
         <v>17</v>
       </c>
@@ -27793,7 +28094,7 @@
         <v>1458</v>
       </c>
     </row>
-    <row r="272" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:24" ht="34" x14ac:dyDescent="0.2">
       <c r="A272" t="s">
         <v>1459</v>
       </c>
@@ -27824,7 +28125,10 @@
       <c r="J272" t="s">
         <v>1461</v>
       </c>
-      <c r="L272" s="6" t="s">
+      <c r="K272" t="s">
+        <v>3936</v>
+      </c>
+      <c r="L272" s="7" t="s">
         <v>1462</v>
       </c>
       <c r="M272" t="s">
@@ -27845,8 +28149,11 @@
       <c r="R272" t="s">
         <v>1464</v>
       </c>
-    </row>
-    <row r="273" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="T272" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="273" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
         <v>1465</v>
       </c>
@@ -27899,7 +28206,7 @@
         <v>1469</v>
       </c>
     </row>
-    <row r="274" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A274" t="s">
         <v>1470</v>
       </c>
@@ -27930,7 +28237,10 @@
       <c r="J274" t="s">
         <v>1472</v>
       </c>
-      <c r="L274" s="6" t="s">
+      <c r="K274" t="s">
+        <v>3937</v>
+      </c>
+      <c r="L274" s="7" t="s">
         <v>1473</v>
       </c>
       <c r="M274" t="s">
@@ -27951,8 +28261,11 @@
       <c r="R274" t="s">
         <v>1474</v>
       </c>
-    </row>
-    <row r="275" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="T274" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="275" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A275" t="s">
         <v>1475</v>
       </c>
@@ -28005,7 +28318,7 @@
         <v>1479</v>
       </c>
     </row>
-    <row r="276" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A276" t="s">
         <v>1480</v>
       </c>
@@ -28036,7 +28349,10 @@
       <c r="J276" t="s">
         <v>1482</v>
       </c>
-      <c r="L276" s="6" t="s">
+      <c r="K276" t="s">
+        <v>3938</v>
+      </c>
+      <c r="L276" s="7" t="s">
         <v>1483</v>
       </c>
       <c r="M276" t="s">
@@ -28057,8 +28373,20 @@
       <c r="R276" t="s">
         <v>1484</v>
       </c>
-    </row>
-    <row r="277" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S276" s="5" t="s">
+        <v>3939</v>
+      </c>
+      <c r="T276" t="s">
+        <v>3869</v>
+      </c>
+      <c r="U276" t="s">
+        <v>3774</v>
+      </c>
+      <c r="V276" t="s">
+        <v>3940</v>
+      </c>
+    </row>
+    <row r="277" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A277" t="s">
         <v>1485</v>
       </c>
@@ -28111,7 +28439,7 @@
         <v>1490</v>
       </c>
     </row>
-    <row r="278" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A278" t="s">
         <v>449</v>
       </c>
@@ -28142,7 +28470,10 @@
       <c r="J278" t="s">
         <v>1491</v>
       </c>
-      <c r="L278" s="6" t="s">
+      <c r="K278" t="s">
+        <v>3941</v>
+      </c>
+      <c r="L278" s="7" t="s">
         <v>1492</v>
       </c>
       <c r="M278" t="s">
@@ -28163,8 +28494,11 @@
       <c r="R278" t="s">
         <v>1494</v>
       </c>
-    </row>
-    <row r="279" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="T278" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="279" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A279" t="s">
         <v>1495</v>
       </c>
@@ -28217,7 +28551,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="280" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A280" t="s">
         <v>449</v>
       </c>
@@ -28248,7 +28582,10 @@
       <c r="J280" t="s">
         <v>1501</v>
       </c>
-      <c r="L280" s="6" t="s">
+      <c r="K280" t="s">
+        <v>3941</v>
+      </c>
+      <c r="L280" s="7" t="s">
         <v>1502</v>
       </c>
       <c r="M280" t="s">
@@ -28269,8 +28606,11 @@
       <c r="R280" t="s">
         <v>1504</v>
       </c>
-    </row>
-    <row r="281" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+      <c r="T280" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="281" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
       <c r="A281" t="s">
         <v>1505</v>
       </c>
@@ -28323,7 +28663,7 @@
         <v>1511</v>
       </c>
     </row>
-    <row r="282" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A282" t="s">
         <v>1512</v>
       </c>
@@ -28354,7 +28694,10 @@
       <c r="J282" t="s">
         <v>1514</v>
       </c>
-      <c r="L282" s="6" t="s">
+      <c r="K282" t="s">
+        <v>3942</v>
+      </c>
+      <c r="L282" s="7" t="s">
         <v>1515</v>
       </c>
       <c r="M282" t="s">
@@ -28375,8 +28718,11 @@
       <c r="R282" t="s">
         <v>1517</v>
       </c>
-    </row>
-    <row r="283" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+      <c r="T282" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="283" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A283" t="s">
         <v>449</v>
       </c>
@@ -28407,7 +28753,10 @@
       <c r="J283" t="s">
         <v>1518</v>
       </c>
-      <c r="L283" s="6" t="s">
+      <c r="K283" t="s">
+        <v>3943</v>
+      </c>
+      <c r="L283" s="7" t="s">
         <v>1519</v>
       </c>
       <c r="M283" t="s">
@@ -28428,8 +28777,11 @@
       <c r="R283" t="s">
         <v>1504</v>
       </c>
-    </row>
-    <row r="284" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+      <c r="T283" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="284" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A284" t="s">
         <v>449</v>
       </c>
@@ -28460,6 +28812,9 @@
       <c r="J284" t="s">
         <v>1520</v>
       </c>
+      <c r="K284" t="s">
+        <v>3943</v>
+      </c>
       <c r="L284" s="6" t="s">
         <v>1521</v>
       </c>
@@ -28481,8 +28836,11 @@
       <c r="R284" t="s">
         <v>1504</v>
       </c>
-    </row>
-    <row r="285" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+      <c r="T284" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="285" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A285" t="s">
         <v>1522</v>
       </c>
@@ -28513,7 +28871,10 @@
       <c r="J285" t="s">
         <v>1524</v>
       </c>
-      <c r="L285" s="6" t="s">
+      <c r="K285" t="s">
+        <v>3944</v>
+      </c>
+      <c r="L285" s="7" t="s">
         <v>1525</v>
       </c>
       <c r="M285" t="s">
@@ -28534,8 +28895,20 @@
       <c r="R285" t="s">
         <v>1526</v>
       </c>
-    </row>
-    <row r="286" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+      <c r="S285" t="s">
+        <v>3945</v>
+      </c>
+      <c r="T285" t="s">
+        <v>3869</v>
+      </c>
+      <c r="U285" t="s">
+        <v>3925</v>
+      </c>
+      <c r="V285" t="s">
+        <v>3946</v>
+      </c>
+    </row>
+    <row r="286" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A286" t="s">
         <v>449</v>
       </c>
@@ -28566,7 +28939,10 @@
       <c r="J286" t="s">
         <v>1527</v>
       </c>
-      <c r="L286" s="6" t="s">
+      <c r="K286" t="s">
+        <v>3943</v>
+      </c>
+      <c r="L286" s="7" t="s">
         <v>1528</v>
       </c>
       <c r="M286" t="s">
@@ -28587,8 +28963,11 @@
       <c r="R286" t="s">
         <v>1504</v>
       </c>
-    </row>
-    <row r="287" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+      <c r="T286" t="s">
+        <v>3868</v>
+      </c>
+    </row>
+    <row r="287" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A287" t="s">
         <v>749</v>
       </c>
@@ -28619,7 +28998,7 @@
       <c r="J287" t="s">
         <v>1529</v>
       </c>
-      <c r="L287" s="6" t="s">
+      <c r="L287" s="7" t="s">
         <v>1530</v>
       </c>
       <c r="M287" t="s">
@@ -28641,7 +29020,7 @@
         <v>1531</v>
       </c>
     </row>
-    <row r="288" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:22" ht="17" x14ac:dyDescent="0.2">
       <c r="A288" t="s">
         <v>754</v>
       </c>
@@ -54803,11 +55182,34 @@
     <hyperlink ref="L214" r:id="rId81" xr:uid="{599864D8-B79C-6643-A7FD-99D6A1E3E455}"/>
     <hyperlink ref="L215" r:id="rId82" xr:uid="{695E64DC-FA59-E646-8C71-B66FD2F35B4E}"/>
     <hyperlink ref="L232" r:id="rId83" xr:uid="{AEF85FA5-5596-3E49-A94A-67E7664387E3}"/>
+    <hyperlink ref="S215" r:id="rId84" xr:uid="{4AD52EC8-B06A-5841-96FA-A822B99D72DC}"/>
+    <hyperlink ref="L234" r:id="rId85" xr:uid="{8ED2110F-45FE-2345-BCBC-744F0BB05AE0}"/>
+    <hyperlink ref="L245" r:id="rId86" xr:uid="{19BE453A-E354-4147-9EBA-B544A4A9BF15}"/>
+    <hyperlink ref="L247" r:id="rId87" xr:uid="{A84A3502-B98D-894D-851C-A07961BD8549}"/>
+    <hyperlink ref="L249" r:id="rId88" xr:uid="{3C9AB634-BE2A-6D45-98AB-CAE3852294ED}"/>
+    <hyperlink ref="L250" r:id="rId89" xr:uid="{E742EE5B-B4F3-AA4F-9EFE-954FC055214E}"/>
+    <hyperlink ref="S250" r:id="rId90" xr:uid="{1DB09AFF-53D5-6947-8587-599E63CB1F71}"/>
+    <hyperlink ref="L259" r:id="rId91" xr:uid="{0F9D0D58-C251-624B-B33C-B470877B8014}"/>
+    <hyperlink ref="S259" r:id="rId92" xr:uid="{34E1A538-A406-1249-9596-ED6B9C20513C}"/>
+    <hyperlink ref="L260" r:id="rId93" xr:uid="{3E8433E6-8418-3349-BA92-A248AB9523DA}"/>
+    <hyperlink ref="L269" r:id="rId94" xr:uid="{4B8716FC-F202-9242-8D12-2941A67CE80E}"/>
+    <hyperlink ref="S269" r:id="rId95" xr:uid="{F28354C8-1435-3C4C-9EEB-92EC6C03CBF2}"/>
+    <hyperlink ref="L272" r:id="rId96" xr:uid="{9E500596-92CE-1443-9346-D7B8C2B9D03F}"/>
+    <hyperlink ref="L274" r:id="rId97" xr:uid="{05A424F1-8284-B646-A9F4-093BB6B6D46B}"/>
+    <hyperlink ref="L276" r:id="rId98" xr:uid="{8A5F73DF-8578-F54E-BB63-4F6A6E51A48E}"/>
+    <hyperlink ref="S276" r:id="rId99" xr:uid="{10A67365-49B1-2A41-8639-62C79595EB17}"/>
+    <hyperlink ref="L278" r:id="rId100" xr:uid="{30B203E5-0FE4-1D4B-B4C2-1A59831168AD}"/>
+    <hyperlink ref="L280" r:id="rId101" xr:uid="{DA2F9BDF-E6F1-8E4D-8607-3F800A253596}"/>
+    <hyperlink ref="L282" r:id="rId102" xr:uid="{8102D2D8-1373-AB43-BC76-54194900E136}"/>
+    <hyperlink ref="L283" r:id="rId103" xr:uid="{F0495F31-ACC7-4F46-93FF-B613C63C5F61}"/>
+    <hyperlink ref="L285" r:id="rId104" xr:uid="{05A56412-360D-714A-9001-7B33791B035A}"/>
+    <hyperlink ref="L286" r:id="rId105" xr:uid="{865B6A08-58FE-6A4F-9841-55DC1FA7B45F}"/>
+    <hyperlink ref="L287" r:id="rId106" xr:uid="{22003204-B4C3-BA4E-A072-4268D31417A4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId84"/>
+    <tablePart r:id="rId107"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>